<commit_message>
pcb rev 1 actually complete (fr this time)
</commit_message>
<xml_diff>
--- a/DRS Project/Design Files/Electrical System/DDR.xlsx
+++ b/DRS Project/Design Files/Electrical System/DDR.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="229">
   <si>
     <t xml:space="preserve">PCB DDR</t>
   </si>
@@ -597,38 +597,52 @@
     <t xml:space="preserve">Completed:</t>
   </si>
   <si>
+    <t xml:space="preserve">YES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewed:</t>
+  </si>
+  <si>
     <t xml:space="preserve">NO</t>
   </si>
   <si>
-    <t xml:space="preserve">Reviewed:</t>
-  </si>
-  <si>
     <t xml:space="preserve">Complete this section before moving to the Schematic Review</t>
   </si>
   <si>
     <t xml:space="preserve">Team Number:</t>
   </si>
   <si>
+    <t xml:space="preserve">DRS Control Unit</t>
+  </si>
+  <si>
     <t xml:space="preserve">Date of DDR:</t>
   </si>
   <si>
     <t xml:space="preserve">PCB Requirements:</t>
   </si>
   <si>
-    <t xml:space="preserve">This should be written to explain the reasoning for having this PCB to someone who is not already familiar with our electric topology.
-E.g. This board is required to receive power from the CEN and distributed it to the cooling system</t>
+    <t xml:space="preserve">This board is required to receive power and a CAN signal from the vehicle/testbench. This board must regulate the power received into voltages appropriate for driving a servo motor and a Teensy 4.0 microcontroller. This board must also communicate with the vehicle/testbench via CAN protocol in order to control a moveable aero device via servo motor.</t>
   </si>
   <si>
     <t xml:space="preserve">Changes from Previous Version:</t>
   </si>
   <si>
+    <t xml:space="preserve">N/A</t>
+  </si>
+  <si>
     <t xml:space="preserve">Top Level Specs</t>
   </si>
   <si>
     <t xml:space="preserve">Input / System Voltage:</t>
   </si>
   <si>
+    <t xml:space="preserve">12-14V</t>
+  </si>
+  <si>
     <t xml:space="preserve">Max Current Draw:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5A</t>
   </si>
   <si>
     <t xml:space="preserve">SCHEMATIC REVIEW</t>
@@ -654,9 +668,6 @@
   </si>
   <si>
     <t xml:space="preserve">Has the ERC been run with no errors?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YES</t>
   </si>
   <si>
     <t xml:space="preserve">Title Block Checklist</t>
@@ -1154,9 +1165,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="30">
     <font>
@@ -1651,20 +1663,24 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="68">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1672,7 +1688,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1680,27 +1696,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1708,47 +1724,47 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1756,11 +1772,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1768,7 +1784,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="2" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1776,7 +1796,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1784,27 +1804,27 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1824,7 +1844,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1836,19 +1856,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1868,7 +1888,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1876,15 +1896,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1892,27 +1912,27 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2793,9 +2813,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2535840</xdr:colOff>
+      <xdr:colOff>2535480</xdr:colOff>
       <xdr:row>65</xdr:row>
-      <xdr:rowOff>104760</xdr:rowOff>
+      <xdr:rowOff>104400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2809,7 +2829,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2009880" y="10265040"/>
-          <a:ext cx="8695800" cy="2707200"/>
+          <a:ext cx="8695440" cy="2706840"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2836,9 +2856,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>3574800</xdr:colOff>
+      <xdr:colOff>3574440</xdr:colOff>
       <xdr:row>73</xdr:row>
-      <xdr:rowOff>55440</xdr:rowOff>
+      <xdr:rowOff>55080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2852,7 +2872,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="811440" y="10121400"/>
-          <a:ext cx="10683000" cy="4196880"/>
+          <a:ext cx="10682640" cy="4196520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3093,438 +3113,438 @@
   <dimension ref="A1:J56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="68.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="68.73"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
+      <c r="B1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
+      <c r="B2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="E5" s="7" t="s">
+      <c r="B5" s="7"/>
+      <c r="E5" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
     </row>
     <row r="8" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="6"/>
+      <c r="B8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="19.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="E9" s="8" t="s">
+      <c r="B9" s="7"/>
+      <c r="E9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
+      <c r="B10" s="7"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
+      <c r="B11" s="7"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="9"/>
+      <c r="B12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="11"/>
+      <c r="B14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="13" t="str">
+      <c r="B15" s="14" t="str">
         <f aca="false">'PCB Design Intent'!B5</f>
-        <v>NO</v>
+        <v>YES</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="13" t="str">
+      <c r="B16" s="14" t="str">
         <f aca="false">'PCB Design Intent'!B6</f>
         <v>NO</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14"/>
-      <c r="B17" s="15"/>
+      <c r="A17" s="15"/>
+      <c r="B17" s="16"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="16"/>
-      <c r="E18" s="8" t="s">
+      <c r="B18" s="17"/>
+      <c r="E18" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="13" t="str">
+      <c r="B19" s="14" t="str">
         <f aca="false">'Schematic Review'!B6</f>
-        <v>NO</v>
-      </c>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
+        <v>YES</v>
+      </c>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="13" t="str">
+      <c r="B20" s="14" t="str">
         <f aca="false">'Schematic Review'!B7</f>
         <v>NO</v>
       </c>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12"/>
-      <c r="B21" s="15"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
+      <c r="A21" s="13"/>
+      <c r="B21" s="16"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="16"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
+      <c r="B22" s="17"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="13" t="str">
+      <c r="B23" s="14" t="str">
         <f aca="false">'Layout Review'!B6</f>
         <v>NO</v>
       </c>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B24" s="13" t="str">
+      <c r="B24" s="14" t="str">
         <f aca="false">'Layout Review'!B7</f>
         <v>NO</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14"/>
-      <c r="B25" s="15"/>
+      <c r="A25" s="15"/>
+      <c r="B25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B26" s="16"/>
+      <c r="B26" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="13" t="str">
+      <c r="B27" s="14" t="str">
         <f aca="false">'Unit Test Checklist'!B5</f>
         <v>NO</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="13" t="str">
+      <c r="B28" s="14" t="str">
         <f aca="false">'Unit Test Checklist'!B6</f>
         <v>NO</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14"/>
-      <c r="B29" s="15"/>
+      <c r="A29" s="15"/>
+      <c r="B29" s="16"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="16" t="s">
+      <c r="A30" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="B30" s="16"/>
+      <c r="B30" s="17"/>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12" t="s">
+      <c r="A31" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="13" t="str">
+      <c r="B31" s="14" t="str">
         <f aca="false">'CAD &amp; Physical Design Review'!B5</f>
         <v>NO</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B32" s="13" t="str">
+      <c r="B32" s="14" t="str">
         <f aca="false">'CAD &amp; Physical Design Review'!B6</f>
         <v>NO</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14"/>
-      <c r="B33" s="15"/>
+      <c r="A33" s="15"/>
+      <c r="B33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17" t="str">
+      <c r="A34" s="18" t="str">
         <f aca="false">IF((AND(B15="YES",B16="YES",B19="YES",B20="YES",B23="YES",B24="YES",B27="YES",B28="YES",B31="YES",B32="YES")), "PCB REVIEWED AND READY FOR MANUFACTURE", "REVIEW NOT COMPLETE")</f>
         <v>REVIEW NOT COMPLETE</v>
       </c>
-      <c r="B34" s="17"/>
+      <c r="B34" s="18"/>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
+      <c r="A37" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B37" s="11"/>
+      <c r="B37" s="12"/>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="18" t="s">
+      <c r="A38" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B38" s="18"/>
+      <c r="B38" s="19"/>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="14"/>
-      <c r="B39" s="15" t="s">
+      <c r="A39" s="15"/>
+      <c r="B39" s="16" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="14"/>
-      <c r="B40" s="15" t="s">
+      <c r="A40" s="15"/>
+      <c r="B40" s="16" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="14"/>
-      <c r="B41" s="15" t="s">
+      <c r="A41" s="15"/>
+      <c r="B41" s="16" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="14"/>
-      <c r="B42" s="15" t="s">
+      <c r="A42" s="15"/>
+      <c r="B42" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="14"/>
-      <c r="B43" s="15" t="s">
+      <c r="A43" s="15"/>
+      <c r="B43" s="16" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="14"/>
-      <c r="B44" s="15" t="s">
+      <c r="A44" s="15"/>
+      <c r="B44" s="16" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="14"/>
-      <c r="B45" s="15" t="s">
+      <c r="A45" s="15"/>
+      <c r="B45" s="16" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="14"/>
-      <c r="B46" s="15" t="s">
+      <c r="A46" s="15"/>
+      <c r="B46" s="16" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="14"/>
-      <c r="B47" s="15" t="s">
+      <c r="A47" s="15"/>
+      <c r="B47" s="16" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="14"/>
-      <c r="B48" s="15" t="s">
+      <c r="A48" s="15"/>
+      <c r="B48" s="16" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="14"/>
-      <c r="B49" s="15" t="s">
+      <c r="A49" s="15"/>
+      <c r="B49" s="16" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="14"/>
-      <c r="B50" s="15" t="s">
+      <c r="A50" s="15"/>
+      <c r="B50" s="16" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="14"/>
-      <c r="B51" s="15" t="s">
+      <c r="A51" s="15"/>
+      <c r="B51" s="16" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="14"/>
-      <c r="B52" s="15" t="s">
+      <c r="A52" s="15"/>
+      <c r="B52" s="16" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="14"/>
-      <c r="B53" s="15" t="s">
+      <c r="A53" s="15"/>
+      <c r="B53" s="16" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="14"/>
-      <c r="B54" s="15" t="s">
+      <c r="A54" s="15"/>
+      <c r="B54" s="16" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="14"/>
-      <c r="B55" s="15" t="s">
+      <c r="A55" s="15"/>
+      <c r="B55" s="16" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="19"/>
-      <c r="B56" s="20" t="s">
+      <c r="A56" s="20"/>
+      <c r="B56" s="21" t="s">
         <v>40</v>
       </c>
     </row>
@@ -3650,155 +3670,165 @@
   <dimension ref="A1:H21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="54.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="54.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30.54"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="2"/>
+      <c r="B1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="3"/>
+      <c r="B2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21"/>
+      <c r="A3" s="22"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="22"/>
+      <c r="B4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="14" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="25" t="s">
-        <v>44</v>
+      <c r="B6" s="26" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21"/>
-      <c r="D7" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
+      <c r="A7" s="22"/>
+      <c r="D7" s="27" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="B8" s="28" t="n">
+      <c r="A8" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="28"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
+      <c r="B9" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="28" t="n">
+      <c r="B10" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="28"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
+      <c r="A11" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="30" t="n">
+        <v>46303</v>
+      </c>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" s="29"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
+      <c r="A13" s="31" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="31"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
     </row>
     <row r="14" customFormat="false" ht="65.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="30" t="s">
-        <v>50</v>
-      </c>
-      <c r="B14" s="30"/>
+      <c r="A14" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="32"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
-        <v>51</v>
+      <c r="A16" s="33" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32"/>
-      <c r="B17" s="32"/>
+      <c r="A17" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="34"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="31" t="s">
-        <v>52</v>
+      <c r="A19" s="33" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="27" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" s="28"/>
+      <c r="A20" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="B21" s="28"/>
+      <c r="A21" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="29" t="s">
+        <v>59</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3847,384 +3877,394 @@
   <dimension ref="A1:E75"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="74.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="33" width="20.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="20.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="74.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="35" width="20.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="60.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="20.73"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="2"/>
+      <c r="A1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="50.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="A2" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="50.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="35" t="s">
-        <v>57</v>
-      </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
+      <c r="A3" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="36"/>
+      <c r="A4" s="22"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="38"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="38"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="40"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="40"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="42"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="43" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="43"/>
+      <c r="D7" s="44"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="22"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="38"/>
+    </row>
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="45" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="45" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="45" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
+    </row>
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="41"/>
-      <c r="D7" s="42"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-    </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="43" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="43" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9" s="43" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="B11" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="C11" s="44"/>
-      <c r="D11" s="45"/>
+      <c r="C11" s="46"/>
+      <c r="D11" s="47"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45"/>
+      <c r="D12" s="45"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
+      <c r="A13" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="46" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
+      <c r="A14" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="46"/>
+      <c r="D14" s="47"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="33"/>
+      <c r="B15" s="35"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="47" t="s">
-        <v>66</v>
-      </c>
-      <c r="B16" s="43"/>
-      <c r="C16" s="43"/>
+      <c r="A16" s="49" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="45"/>
+      <c r="C16" s="45"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="46" t="s">
-        <v>67</v>
-      </c>
-      <c r="B17" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" s="44"/>
-      <c r="D17" s="45"/>
+      <c r="A17" s="48" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="46"/>
+      <c r="D17" s="47"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="46" t="s">
-        <v>68</v>
-      </c>
-      <c r="B18" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="C18" s="44"/>
-      <c r="D18" s="45"/>
+      <c r="A18" s="48" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="46"/>
+      <c r="D18" s="47"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="46" t="s">
-        <v>69</v>
-      </c>
-      <c r="B19" s="44"/>
-      <c r="C19" s="44"/>
-      <c r="D19" s="45"/>
+      <c r="A19" s="48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="46"/>
+      <c r="D19" s="47"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="46" t="s">
-        <v>70</v>
-      </c>
-      <c r="B20" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="C20" s="44"/>
-      <c r="D20" s="45"/>
+      <c r="A20" s="48" t="s">
+        <v>74</v>
+      </c>
+      <c r="B20" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="46"/>
+      <c r="D20" s="47"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="46" t="s">
-        <v>71</v>
-      </c>
-      <c r="B21" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="C21" s="44"/>
-      <c r="D21" s="45"/>
+      <c r="A21" s="48" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="46"/>
+      <c r="D21" s="47"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="46" t="s">
-        <v>72</v>
-      </c>
-      <c r="B22" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="C22" s="44"/>
-      <c r="D22" s="45"/>
+      <c r="A22" s="48" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="46"/>
+      <c r="D22" s="47"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="46" t="s">
-        <v>73</v>
-      </c>
-      <c r="B23" s="44"/>
-      <c r="C23" s="44"/>
-      <c r="D23" s="45"/>
+      <c r="A23" s="48" t="s">
+        <v>77</v>
+      </c>
+      <c r="B23" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="46"/>
+      <c r="D23" s="47"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="46"/>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="46"/>
+      <c r="A24" s="48"/>
+      <c r="B24" s="48"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="48"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="46"/>
+      <c r="A25" s="48"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="47" t="s">
-        <v>74</v>
-      </c>
-      <c r="B26" s="43"/>
-      <c r="C26" s="43"/>
+      <c r="A26" s="49" t="s">
+        <v>78</v>
+      </c>
+      <c r="B26" s="45"/>
+      <c r="C26" s="45"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="46" t="s">
-        <v>75</v>
-      </c>
-      <c r="B27" s="44"/>
-      <c r="C27" s="44"/>
-      <c r="D27" s="45"/>
+      <c r="A27" s="48" t="s">
+        <v>79</v>
+      </c>
+      <c r="B27" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="46"/>
+      <c r="D27" s="47"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="33"/>
+      <c r="B28" s="35"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="47" t="s">
-        <v>76</v>
-      </c>
-      <c r="B29" s="48"/>
-      <c r="C29" s="48"/>
+      <c r="A29" s="49" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="50"/>
+      <c r="C29" s="50"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="46" t="s">
-        <v>77</v>
-      </c>
-      <c r="B30" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="C30" s="44"/>
-      <c r="D30" s="45"/>
+      <c r="A30" s="48" t="s">
+        <v>81</v>
+      </c>
+      <c r="B30" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" s="46"/>
+      <c r="D30" s="47"/>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="46" t="s">
-        <v>78</v>
-      </c>
-      <c r="B31" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="C31" s="44"/>
-      <c r="D31" s="45"/>
+      <c r="A31" s="48" t="s">
+        <v>82</v>
+      </c>
+      <c r="B31" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C31" s="46"/>
+      <c r="D31" s="47"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="33"/>
+      <c r="B32" s="35"/>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="47" t="s">
-        <v>79</v>
-      </c>
-      <c r="B33" s="48"/>
-      <c r="C33" s="48"/>
+      <c r="A33" s="49" t="s">
+        <v>83</v>
+      </c>
+      <c r="B33" s="50"/>
+      <c r="C33" s="50"/>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="46" t="s">
-        <v>80</v>
-      </c>
-      <c r="B34" s="44" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34" s="44"/>
-      <c r="D34" s="45"/>
+      <c r="A34" s="48" t="s">
+        <v>84</v>
+      </c>
+      <c r="B34" s="46" t="s">
+        <v>85</v>
+      </c>
+      <c r="C34" s="46"/>
+      <c r="D34" s="47"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="46" t="s">
-        <v>82</v>
-      </c>
-      <c r="B35" s="44" t="s">
-        <v>81</v>
-      </c>
-      <c r="C35" s="44"/>
-      <c r="D35" s="45"/>
+      <c r="A35" s="48" t="s">
+        <v>86</v>
+      </c>
+      <c r="B35" s="46" t="s">
+        <v>85</v>
+      </c>
+      <c r="C35" s="46"/>
+      <c r="D35" s="47"/>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="B36" s="44" t="s">
-        <v>81</v>
-      </c>
-      <c r="C36" s="44"/>
-      <c r="D36" s="45"/>
+      <c r="A36" s="48" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="46" t="s">
+        <v>85</v>
+      </c>
+      <c r="C36" s="46"/>
+      <c r="D36" s="47"/>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="46" t="s">
-        <v>84</v>
-      </c>
-      <c r="B37" s="44" t="s">
+      <c r="A37" s="48" t="s">
+        <v>88</v>
+      </c>
+      <c r="B37" s="46" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37" s="46"/>
+      <c r="D37" s="47"/>
+    </row>
+    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="48" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" s="46" t="s">
         <v>85</v>
       </c>
-      <c r="C37" s="44"/>
-      <c r="D37" s="45"/>
-    </row>
-    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="46" t="s">
-        <v>86</v>
-      </c>
-      <c r="B38" s="44"/>
-      <c r="C38" s="44"/>
-      <c r="D38" s="45"/>
+      <c r="C38" s="46"/>
+      <c r="D38" s="47"/>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="46" t="s">
-        <v>87</v>
-      </c>
-      <c r="B39" s="44" t="s">
-        <v>81</v>
-      </c>
-      <c r="C39" s="44"/>
-      <c r="D39" s="45"/>
+      <c r="A39" s="48" t="s">
+        <v>91</v>
+      </c>
+      <c r="B39" s="46" t="s">
+        <v>85</v>
+      </c>
+      <c r="C39" s="46"/>
+      <c r="D39" s="47"/>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="33"/>
+      <c r="B40" s="35"/>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="47" t="s">
-        <v>88</v>
-      </c>
-      <c r="B41" s="33"/>
+      <c r="A41" s="49" t="s">
+        <v>92</v>
+      </c>
+      <c r="B41" s="35"/>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="46" t="s">
-        <v>89</v>
-      </c>
-      <c r="B42" s="44"/>
-      <c r="C42" s="44"/>
-      <c r="D42" s="45"/>
+      <c r="A42" s="48" t="s">
+        <v>93</v>
+      </c>
+      <c r="B42" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C42" s="46"/>
+      <c r="D42" s="47"/>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="49" t="s">
-        <v>90</v>
-      </c>
-      <c r="B43" s="50" t="s">
-        <v>63</v>
-      </c>
-      <c r="C43" s="50"/>
-      <c r="D43" s="51"/>
+      <c r="A43" s="51" t="s">
+        <v>94</v>
+      </c>
+      <c r="B43" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="C43" s="52"/>
+      <c r="D43" s="53"/>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="33"/>
+      <c r="B44" s="35"/>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
+      <c r="A46" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="B46" s="9"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="8"/>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
+      <c r="A47" s="9"/>
+      <c r="B47" s="9"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="8"/>
-      <c r="B48" s="8"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
+      <c r="A48" s="9"/>
+      <c r="B48" s="9"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="8"/>
-      <c r="B49" s="8"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
+      <c r="A49" s="9"/>
+      <c r="B49" s="9"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E75" s="0" t="s">
-        <v>92</v>
+      <c r="E75" s="1" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -4343,316 +4383,316 @@
   <dimension ref="A1:F58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="33" width="20.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="20.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="72.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="35" width="20.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="60.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="20.73"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="2"/>
+      <c r="A1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="51" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="A2" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="51" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
+      <c r="A3" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
     </row>
     <row r="4" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="36"/>
+      <c r="A4" s="22"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="38"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="38"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="40"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="39" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="52"/>
+      <c r="B6" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="41"/>
+      <c r="D6" s="54"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="41" t="s">
-        <v>44</v>
-      </c>
-      <c r="C7" s="41"/>
-      <c r="D7" s="53"/>
+      <c r="B7" s="43" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="43"/>
+      <c r="D7" s="55"/>
     </row>
     <row r="8" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21"/>
-      <c r="B8" s="21"/>
-      <c r="C8" s="36"/>
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="38"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="43" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="43" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9" s="43" t="s">
-        <v>60</v>
+      <c r="B9" s="45" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="45" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="45" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="B10" s="31"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
+      <c r="A10" s="33" t="s">
+        <v>100</v>
+      </c>
+      <c r="B10" s="33"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="46" t="s">
-        <v>97</v>
-      </c>
-      <c r="B11" s="44"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="45"/>
+      <c r="A11" s="48" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" s="46"/>
+      <c r="C11" s="46"/>
+      <c r="D11" s="47"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
+      <c r="A13" s="33" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="54" t="s">
-        <v>99</v>
-      </c>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
+      <c r="A14" s="56" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="46"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="47"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C15" s="43"/>
-      <c r="D15" s="43"/>
+      <c r="C15" s="45"/>
+      <c r="D15" s="45"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="B16" s="31"/>
-      <c r="C16" s="43"/>
-      <c r="D16" s="43"/>
+      <c r="A16" s="33" t="s">
+        <v>104</v>
+      </c>
+      <c r="B16" s="33"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="45"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="46" t="s">
-        <v>101</v>
-      </c>
-      <c r="B17" s="44"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="45"/>
+      <c r="A17" s="48" t="s">
+        <v>105</v>
+      </c>
+      <c r="B17" s="46"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="47"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="46" t="s">
-        <v>102</v>
-      </c>
-      <c r="B18" s="44"/>
-      <c r="C18" s="44"/>
-      <c r="D18" s="45"/>
+      <c r="A18" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="B18" s="46"/>
+      <c r="C18" s="46"/>
+      <c r="D18" s="47"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="B19" s="44"/>
-      <c r="C19" s="44"/>
-      <c r="D19" s="45"/>
+      <c r="A19" s="48" t="s">
+        <v>107</v>
+      </c>
+      <c r="B19" s="46"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="47"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="46" t="s">
-        <v>104</v>
-      </c>
-      <c r="B20" s="44"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="45"/>
+      <c r="A20" s="48" t="s">
+        <v>108</v>
+      </c>
+      <c r="B20" s="46"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="47"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="B21" s="44"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="45"/>
+      <c r="A21" s="48" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" s="46"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="47"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="47" t="s">
-        <v>106</v>
-      </c>
-      <c r="B23" s="47"/>
-      <c r="C23" s="43"/>
+      <c r="A23" s="49" t="s">
+        <v>110</v>
+      </c>
+      <c r="B23" s="49"/>
+      <c r="C23" s="45"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="46" t="s">
-        <v>107</v>
-      </c>
-      <c r="B24" s="44"/>
-      <c r="C24" s="44"/>
-      <c r="D24" s="45"/>
+      <c r="A24" s="48" t="s">
+        <v>111</v>
+      </c>
+      <c r="B24" s="46"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="47"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="46" t="s">
-        <v>108</v>
-      </c>
-      <c r="B25" s="44"/>
-      <c r="C25" s="44"/>
-      <c r="D25" s="45"/>
+      <c r="A25" s="48" t="s">
+        <v>112</v>
+      </c>
+      <c r="B25" s="46"/>
+      <c r="C25" s="46"/>
+      <c r="D25" s="47"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="46" t="s">
-        <v>109</v>
-      </c>
-      <c r="B26" s="44"/>
-      <c r="C26" s="44"/>
-      <c r="D26" s="45"/>
+      <c r="A26" s="48" t="s">
+        <v>113</v>
+      </c>
+      <c r="B26" s="46"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="47"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="B27" s="44"/>
-      <c r="C27" s="44"/>
-      <c r="D27" s="45"/>
+      <c r="A27" s="48" t="s">
+        <v>114</v>
+      </c>
+      <c r="B27" s="46"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="47"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="46" t="s">
-        <v>111</v>
-      </c>
-      <c r="B28" s="44"/>
-      <c r="C28" s="44"/>
-      <c r="D28" s="45"/>
+      <c r="A28" s="48" t="s">
+        <v>115</v>
+      </c>
+      <c r="B28" s="46"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="47"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="0" t="s">
-        <v>112</v>
+      <c r="B29" s="1" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="47" t="s">
-        <v>113</v>
-      </c>
-      <c r="B30" s="47"/>
-      <c r="C30" s="48"/>
+      <c r="A30" s="49" t="s">
+        <v>117</v>
+      </c>
+      <c r="B30" s="49"/>
+      <c r="C30" s="50"/>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="46" t="s">
-        <v>114</v>
-      </c>
-      <c r="B31" s="44"/>
-      <c r="C31" s="44"/>
-      <c r="D31" s="45"/>
+      <c r="A31" s="48" t="s">
+        <v>118</v>
+      </c>
+      <c r="B31" s="46"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="47"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="46" t="s">
-        <v>115</v>
-      </c>
-      <c r="B32" s="44"/>
-      <c r="C32" s="44"/>
-      <c r="D32" s="45"/>
+      <c r="A32" s="48" t="s">
+        <v>119</v>
+      </c>
+      <c r="B32" s="46"/>
+      <c r="C32" s="46"/>
+      <c r="D32" s="47"/>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="46" t="s">
-        <v>116</v>
-      </c>
-      <c r="B33" s="44"/>
-      <c r="C33" s="44"/>
-      <c r="D33" s="45"/>
+      <c r="A33" s="48" t="s">
+        <v>120</v>
+      </c>
+      <c r="B33" s="46"/>
+      <c r="C33" s="46"/>
+      <c r="D33" s="47"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="47" t="s">
-        <v>117</v>
-      </c>
-      <c r="B35" s="48"/>
-      <c r="C35" s="48"/>
+      <c r="A35" s="49" t="s">
+        <v>121</v>
+      </c>
+      <c r="B35" s="50"/>
+      <c r="C35" s="50"/>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="46" t="s">
-        <v>118</v>
-      </c>
-      <c r="B36" s="44"/>
-      <c r="C36" s="44"/>
-      <c r="D36" s="45"/>
+      <c r="A36" s="48" t="s">
+        <v>122</v>
+      </c>
+      <c r="B36" s="46"/>
+      <c r="C36" s="46"/>
+      <c r="D36" s="47"/>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="46" t="s">
-        <v>119</v>
-      </c>
-      <c r="B37" s="44"/>
-      <c r="C37" s="44"/>
-      <c r="D37" s="45"/>
+      <c r="A37" s="48" t="s">
+        <v>123</v>
+      </c>
+      <c r="B37" s="46"/>
+      <c r="C37" s="46"/>
+      <c r="D37" s="47"/>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="46" t="s">
-        <v>120</v>
-      </c>
-      <c r="B38" s="44"/>
-      <c r="C38" s="44"/>
-      <c r="D38" s="45"/>
+      <c r="A38" s="48" t="s">
+        <v>124</v>
+      </c>
+      <c r="B38" s="46"/>
+      <c r="C38" s="46"/>
+      <c r="D38" s="47"/>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="46" t="s">
-        <v>121</v>
-      </c>
-      <c r="B39" s="44"/>
-      <c r="C39" s="44"/>
-      <c r="D39" s="45"/>
+      <c r="A39" s="48" t="s">
+        <v>125</v>
+      </c>
+      <c r="B39" s="46"/>
+      <c r="C39" s="46"/>
+      <c r="D39" s="47"/>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
+      <c r="B42" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="8"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="8"/>
+      <c r="B43" s="9"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
+      <c r="B44" s="9"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
+      <c r="B45" s="9"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F58" s="0" t="s">
-        <v>123</v>
+      <c r="F58" s="1" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -4753,175 +4793,175 @@
   <dimension ref="A1:D27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="67.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="33" width="20.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="20.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="67.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="35" width="20.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="60.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="20.73"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="2"/>
+      <c r="A1" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="51" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="A2" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21"/>
-      <c r="B3" s="21"/>
-      <c r="C3" s="36"/>
+      <c r="A3" s="22"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="38"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="38"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="40"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="39" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="39"/>
-      <c r="D5" s="52"/>
+      <c r="B5" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="41"/>
+      <c r="D5" s="54"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="41" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="41"/>
-      <c r="D6" s="53"/>
+      <c r="B6" s="43" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="43"/>
+      <c r="D6" s="55"/>
     </row>
     <row r="7" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
+      <c r="A7" s="22"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="38"/>
     </row>
     <row r="8" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
+      <c r="A8" s="22"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="38"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="43" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="43" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9" s="43" t="s">
-        <v>60</v>
+      <c r="B9" s="45" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="45" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="45" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
-        <v>126</v>
-      </c>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
+      <c r="A10" s="33" t="s">
+        <v>130</v>
+      </c>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="B11" s="44"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="55"/>
+      <c r="A11" s="48" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" s="46"/>
+      <c r="C11" s="46"/>
+      <c r="D11" s="57"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="46" t="s">
-        <v>128</v>
-      </c>
-      <c r="B12" s="44"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="55"/>
+      <c r="A12" s="48" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" s="46"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="57"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="46" t="s">
-        <v>129</v>
-      </c>
-      <c r="B13" s="44"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="55"/>
+      <c r="A13" s="48" t="s">
+        <v>133</v>
+      </c>
+      <c r="B13" s="46"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="57"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="46" t="s">
-        <v>130</v>
-      </c>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="55"/>
+      <c r="A14" s="48" t="s">
+        <v>134</v>
+      </c>
+      <c r="B14" s="46"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="57"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="33"/>
+      <c r="B15" s="35"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="47" t="s">
-        <v>131</v>
-      </c>
-      <c r="B16" s="43"/>
-      <c r="C16" s="43"/>
+      <c r="A16" s="49" t="s">
+        <v>135</v>
+      </c>
+      <c r="B16" s="45"/>
+      <c r="C16" s="45"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="46" t="s">
-        <v>132</v>
-      </c>
-      <c r="B17" s="44"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="55"/>
+      <c r="A17" s="48" t="s">
+        <v>136</v>
+      </c>
+      <c r="B17" s="46"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="57"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="46" t="s">
-        <v>133</v>
-      </c>
-      <c r="B18" s="44"/>
-      <c r="C18" s="44"/>
-      <c r="D18" s="55"/>
+      <c r="A18" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="B18" s="46"/>
+      <c r="C18" s="46"/>
+      <c r="D18" s="57"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="31" t="s">
-        <v>134</v>
+      <c r="A20" s="33" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="46" t="s">
-        <v>135</v>
-      </c>
-      <c r="B21" s="44"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="55"/>
+      <c r="A21" s="48" t="s">
+        <v>139</v>
+      </c>
+      <c r="B21" s="46"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="57"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="46" t="s">
-        <v>136</v>
-      </c>
-      <c r="B22" s="44"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="55"/>
+      <c r="A22" s="48" t="s">
+        <v>140</v>
+      </c>
+      <c r="B22" s="46"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="57"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="0" t="s">
-        <v>112</v>
+      <c r="B27" s="1" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -4987,276 +5027,276 @@
   <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="31.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="121.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="42.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="31.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="121.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="42.27"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="A1" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="56" t="s">
-        <v>138</v>
-      </c>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
+      <c r="A2" s="58" t="s">
+        <v>142</v>
+      </c>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="57"/>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
+      <c r="A3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="38"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="40"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="52"/>
+      <c r="B5" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="54"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="59" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="53"/>
+      <c r="B6" s="61" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="55"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="57"/>
-      <c r="B7" s="58"/>
-      <c r="C7" s="58"/>
-      <c r="D7" s="58"/>
-      <c r="E7" s="58"/>
-      <c r="F7" s="58"/>
-      <c r="G7" s="58"/>
+      <c r="A7" s="59"/>
+      <c r="B7" s="60"/>
+      <c r="C7" s="60"/>
+      <c r="D7" s="60"/>
+      <c r="E7" s="60"/>
+      <c r="F7" s="60"/>
+      <c r="G7" s="60"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="60" t="s">
-        <v>139</v>
-      </c>
-      <c r="B9" s="60" t="s">
-        <v>140</v>
-      </c>
-      <c r="C9" s="60" t="s">
-        <v>141</v>
-      </c>
-      <c r="D9" s="60" t="s">
-        <v>142</v>
-      </c>
-      <c r="E9" s="60" t="s">
+      <c r="A9" s="62" t="s">
         <v>143</v>
       </c>
-      <c r="F9" s="60" t="s">
+      <c r="B9" s="62" t="s">
         <v>144</v>
       </c>
-      <c r="G9" s="60" t="s">
+      <c r="C9" s="62" t="s">
         <v>145</v>
       </c>
+      <c r="D9" s="62" t="s">
+        <v>146</v>
+      </c>
+      <c r="E9" s="62" t="s">
+        <v>147</v>
+      </c>
+      <c r="F9" s="62" t="s">
+        <v>148</v>
+      </c>
+      <c r="G9" s="62" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="60" t="s">
-        <v>146</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="D10" s="60" t="s">
-        <v>149</v>
-      </c>
-      <c r="E10" s="0" t="s">
+      <c r="A10" s="62" t="s">
         <v>150</v>
       </c>
+      <c r="B10" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D10" s="62" t="s">
+        <v>153</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="60" t="s">
-        <v>151</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="C11" s="0" t="s">
+      <c r="A11" s="62" t="s">
+        <v>155</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D11" s="62" t="s">
+        <v>158</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E12" s="63" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="D11" s="60" t="s">
-        <v>154</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="C12" s="0" t="s">
+      <c r="E13" s="63" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="D12" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="E12" s="61" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>151</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="E13" s="61" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="B14" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="C14" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="E14" s="61" t="s">
-        <v>165</v>
+      <c r="E14" s="63" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="60" t="s">
-        <v>166</v>
-      </c>
-      <c r="B15" s="0" t="s">
-        <v>167</v>
-      </c>
-      <c r="C15" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="D15" s="60" t="s">
-        <v>149</v>
-      </c>
-      <c r="E15" s="0" t="s">
-        <v>169</v>
+      <c r="A15" s="62" t="s">
+        <v>170</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="D15" s="62" t="s">
+        <v>153</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="B16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C16" s="0" t="s">
-        <v>171</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="E16" s="61" t="s">
-        <v>172</v>
+      <c r="B16" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E16" s="63" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="B17" s="0" t="s">
-        <v>173</v>
-      </c>
-      <c r="C17" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="D17" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="E17" s="61" t="s">
-        <v>175</v>
+      <c r="A17" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E17" s="63" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
-        <v>176</v>
-      </c>
-      <c r="B18" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="C18" s="0" t="s">
-        <v>178</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="E18" s="61" t="s">
-        <v>179</v>
+      <c r="A18" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E18" s="63" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
-        <v>180</v>
-      </c>
-      <c r="B19" s="0" t="s">
-        <v>181</v>
-      </c>
-      <c r="C19" s="0" t="s">
-        <v>182</v>
-      </c>
-      <c r="D19" s="0" t="s">
-        <v>183</v>
-      </c>
-      <c r="E19" s="61" t="s">
+      <c r="A19" s="1" t="s">
         <v>184</v>
       </c>
+      <c r="B19" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E19" s="63" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E20" s="62" t="s">
-        <v>185</v>
+      <c r="E20" s="64" t="s">
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -5317,79 +5357,79 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="65.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="67.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="71.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="65.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="67.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="71.45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="A1" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="63" t="s">
-        <v>187</v>
-      </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
+      <c r="A2" s="65" t="s">
+        <v>191</v>
+      </c>
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="38"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="40"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="52"/>
+      <c r="B5" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="54"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="59" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="53"/>
+      <c r="B6" s="61" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="55"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="60" t="s">
-        <v>188</v>
-      </c>
-      <c r="B9" s="60" t="s">
-        <v>189</v>
-      </c>
-      <c r="C9" s="60" t="s">
-        <v>190</v>
-      </c>
-      <c r="D9" s="60" t="s">
-        <v>191</v>
+      <c r="A9" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="B9" s="62" t="s">
+        <v>193</v>
+      </c>
+      <c r="C9" s="62" t="s">
+        <v>194</v>
+      </c>
+      <c r="D9" s="62" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="64" t="n">
+      <c r="A10" s="66" t="n">
         <v>36526</v>
       </c>
-      <c r="B10" s="0" t="s">
-        <v>192</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>193</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>194</v>
+      <c r="B10" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -5438,170 +5478,170 @@
   <dimension ref="A1:J8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="23.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="57.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="26.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="21.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="57.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="26.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="22.18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="31" t="s">
-        <v>195</v>
-      </c>
-      <c r="B1" s="31" t="s">
-        <v>196</v>
-      </c>
-      <c r="C1" s="31" t="s">
-        <v>197</v>
-      </c>
-      <c r="D1" s="31" t="s">
-        <v>198</v>
-      </c>
-      <c r="E1" s="60" t="s">
-        <v>139</v>
-      </c>
-      <c r="F1" s="60" t="s">
+      <c r="A1" s="33" t="s">
         <v>199</v>
       </c>
-      <c r="G1" s="60" t="s">
+      <c r="B1" s="33" t="s">
         <v>200</v>
       </c>
-      <c r="H1" s="60" t="s">
+      <c r="C1" s="33" t="s">
         <v>201</v>
       </c>
-      <c r="I1" s="60" t="s">
+      <c r="D1" s="33" t="s">
         <v>202</v>
       </c>
-      <c r="J1" s="60" t="s">
+      <c r="E1" s="62" t="s">
+        <v>143</v>
+      </c>
+      <c r="F1" s="62" t="s">
         <v>203</v>
       </c>
+      <c r="G1" s="62" t="s">
+        <v>204</v>
+      </c>
+      <c r="H1" s="62" t="s">
+        <v>205</v>
+      </c>
+      <c r="I1" s="62" t="s">
+        <v>206</v>
+      </c>
+      <c r="J1" s="62" t="s">
+        <v>207</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="65" t="s">
-        <v>63</v>
-      </c>
-      <c r="B2" s="65" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>204</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>205</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>206</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>146</v>
-      </c>
-      <c r="G2" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="H2" s="0" t="s">
-        <v>207</v>
-      </c>
-      <c r="I2" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="J2" s="0" t="s">
+      <c r="A2" s="67" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="67" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>208</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="65" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="65" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>209</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>210</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>211</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>151</v>
-      </c>
-      <c r="G3" s="0" t="s">
-        <v>212</v>
-      </c>
-      <c r="H3" s="0" t="s">
+      <c r="A3" s="67" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="67" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="J3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>215</v>
       </c>
+      <c r="F3" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="65" t="s">
-        <v>216</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>217</v>
-      </c>
-      <c r="E4" s="0" t="s">
-        <v>218</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="G4" s="0" t="s">
-        <v>183</v>
-      </c>
-      <c r="I4" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="J4" s="0" t="s">
-        <v>219</v>
+      <c r="B4" s="67" t="s">
+        <v>220</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="0" t="s">
-        <v>220</v>
-      </c>
-      <c r="E5" s="0" t="s">
-        <v>221</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="G5" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="J5" s="0" t="s">
-        <v>222</v>
+      <c r="C5" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F6" s="0" t="s">
-        <v>223</v>
-      </c>
-      <c r="J6" s="0" t="s">
-        <v>224</v>
+      <c r="F6" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F7" s="0" t="s">
-        <v>176</v>
+      <c r="F7" s="1" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F8" s="0" t="s">
-        <v>180</v>
+      <c r="F8" s="1" t="s">
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
made minor changes to pcb and *nearly* finished
</commit_message>
<xml_diff>
--- a/DRS Project/Design Files/Electrical System/DDR.xlsx
+++ b/DRS Project/Design Files/Electrical System/DDR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/theodevos-vernes/Documents/GitHub/ENGG2200/DRS Project/Design Files/Electrical System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C9E6D7E-02AD-C74C-AAAF-8B92180D9581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4D9C421-AE1D-5E4C-BC6C-C313A2E733C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DETAILED DESIGN REVIEW" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="229">
   <si>
     <t>PCB DDR</t>
   </si>
@@ -1175,18 +1175,6 @@
   </si>
   <si>
     <t>Element14</t>
-  </si>
-  <si>
-    <t>Issues with Deutsch connector footprint</t>
-  </si>
-  <si>
-    <t>???</t>
-  </si>
-  <si>
-    <t>What locking tabs? N/A?</t>
-  </si>
-  <si>
-    <t>I believe so, check with Adam</t>
   </si>
 </sst>
 </file>
@@ -1334,14 +1322,14 @@
       <sz val="20"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="20"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1709,45 +1697,6 @@
   </cellStyleXfs>
   <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="18" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="16" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1841,6 +1790,48 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="16" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="18" xfId="2" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="2" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1852,9 +1843,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="2" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="2" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -3058,446 +3046,440 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
+      <c r="B1" s="2"/>
     </row>
     <row r="2" spans="1:10" ht="80.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="13"/>
+      <c r="B2" s="47"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="56"/>
     </row>
     <row r="4" spans="1:10" ht="21" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
     </row>
     <row r="5" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="57"/>
+      <c r="I5" s="57"/>
+      <c r="J5" s="57"/>
     </row>
     <row r="6" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="4">
         <v>1</v>
       </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
+      <c r="G6" s="57"/>
+      <c r="H6" s="57"/>
+      <c r="I6" s="57"/>
+      <c r="J6" s="57"/>
     </row>
     <row r="8" spans="1:10" ht="21" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="17"/>
+      <c r="B8" s="4"/>
     </row>
     <row r="9" spans="1:10" ht="19.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="E9" s="8" t="s">
+      <c r="B9" s="4"/>
+      <c r="E9" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="46"/>
+      <c r="J9" s="46"/>
     </row>
     <row r="10" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
+      <c r="B10" s="4"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="46"/>
+      <c r="J10" s="46"/>
     </row>
     <row r="11" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
+      <c r="B11" s="4"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="46"/>
+      <c r="I11" s="46"/>
+      <c r="J11" s="46"/>
     </row>
     <row r="12" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="5"/>
+      <c r="B12" s="58"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="18"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="4"/>
+      <c r="B14" s="54"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="20" t="str">
+      <c r="B15" s="7" t="str">
         <f>'PCB Design Intent'!B5</f>
         <v>YES</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="20" t="str">
+      <c r="B16" s="7" t="str">
         <f>'PCB Design Intent'!B6</f>
         <v>NO</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="21"/>
-      <c r="B17" s="22"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="9"/>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="3"/>
-      <c r="E18" s="8" t="s">
+      <c r="B18" s="52"/>
+      <c r="E18" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="46"/>
+      <c r="I18" s="46"/>
+      <c r="J18" s="46"/>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="20" t="str">
+      <c r="B19" s="7" t="str">
         <f>'Schematic Review'!B6</f>
         <v>YES</v>
       </c>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="46"/>
     </row>
     <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="20" t="str">
+      <c r="B20" s="7" t="str">
         <f>'Schematic Review'!B7</f>
         <v>NO</v>
       </c>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
+      <c r="E20" s="46"/>
+      <c r="F20" s="46"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="46"/>
+      <c r="I20" s="46"/>
+      <c r="J20" s="46"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" s="19"/>
-      <c r="B21" s="22"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
+      <c r="A21" s="6"/>
+      <c r="B21" s="9"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="46"/>
+      <c r="J21" s="46"/>
     </row>
     <row r="22" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="3"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
+      <c r="B22" s="52"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="46"/>
+      <c r="H22" s="46"/>
+      <c r="I22" s="46"/>
+      <c r="J22" s="46"/>
     </row>
     <row r="23" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="20" t="str">
+      <c r="B23" s="7" t="str">
         <f>'Layout Review'!B6</f>
         <v>NO</v>
       </c>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
+      <c r="I23" s="46"/>
+      <c r="J23" s="46"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B24" s="20" t="str">
+      <c r="B24" s="7" t="str">
         <f>'Layout Review'!B7</f>
         <v>NO</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="21"/>
-      <c r="B25" s="22"/>
+      <c r="A25" s="8"/>
+      <c r="B25" s="9"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="B26" s="3"/>
+      <c r="B26" s="52"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="20" t="str">
+      <c r="B27" s="7" t="str">
         <f>'Unit Test Checklist'!B5</f>
         <v>NO</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="20" t="str">
+      <c r="B28" s="7" t="str">
         <f>'Unit Test Checklist'!B6</f>
         <v>NO</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="21"/>
-      <c r="B29" s="22"/>
+      <c r="A29" s="8"/>
+      <c r="B29" s="9"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="B30" s="3"/>
+      <c r="B30" s="52"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A31" s="19" t="s">
+      <c r="A31" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="20" t="str">
+      <c r="B31" s="7" t="str">
         <f>'CAD &amp; Physical Design Review'!B5</f>
         <v>NO</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A32" s="19" t="s">
+      <c r="A32" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B32" s="20" t="str">
+      <c r="B32" s="7" t="str">
         <f>'CAD &amp; Physical Design Review'!B6</f>
         <v>NO</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" s="21"/>
-      <c r="B33" s="22"/>
+      <c r="A33" s="8"/>
+      <c r="B33" s="9"/>
     </row>
     <row r="34" spans="1:2" ht="26" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="str">
+      <c r="A34" s="53" t="str">
         <f>IF((AND(B15="YES",B16="YES",B19="YES",B20="YES",B23="YES",B24="YES",B27="YES",B28="YES",B31="YES",B32="YES")), "PCB REVIEWED AND READY FOR MANUFACTURE", "REVIEW NOT COMPLETE")</f>
         <v>REVIEW NOT COMPLETE</v>
       </c>
-      <c r="B34" s="2"/>
+      <c r="B34" s="53"/>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="B37" s="4"/>
+      <c r="B37" s="54"/>
     </row>
     <row r="38" spans="1:2" ht="23.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
+      <c r="A38" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="B38" s="1"/>
+      <c r="B38" s="55"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A39" s="21"/>
-      <c r="B39" s="22" t="s">
+      <c r="A39" s="8"/>
+      <c r="B39" s="9" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A40" s="21"/>
-      <c r="B40" s="22" t="s">
+      <c r="A40" s="8"/>
+      <c r="B40" s="9" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A41" s="21"/>
-      <c r="B41" s="22" t="s">
+      <c r="A41" s="8"/>
+      <c r="B41" s="9" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" s="21"/>
-      <c r="B42" s="22" t="s">
+      <c r="A42" s="8"/>
+      <c r="B42" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" s="21"/>
-      <c r="B43" s="22" t="s">
+      <c r="A43" s="8"/>
+      <c r="B43" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A44" s="21"/>
-      <c r="B44" s="22" t="s">
+      <c r="A44" s="8"/>
+      <c r="B44" s="9" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A45" s="21"/>
-      <c r="B45" s="22" t="s">
+      <c r="A45" s="8"/>
+      <c r="B45" s="9" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A46" s="21"/>
-      <c r="B46" s="22" t="s">
+      <c r="A46" s="8"/>
+      <c r="B46" s="9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A47" s="21"/>
-      <c r="B47" s="22" t="s">
+      <c r="A47" s="8"/>
+      <c r="B47" s="9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A48" s="21"/>
-      <c r="B48" s="22" t="s">
+      <c r="A48" s="8"/>
+      <c r="B48" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A49" s="21"/>
-      <c r="B49" s="22" t="s">
+      <c r="A49" s="8"/>
+      <c r="B49" s="9" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A50" s="21"/>
-      <c r="B50" s="22" t="s">
+      <c r="A50" s="8"/>
+      <c r="B50" s="9" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A51" s="21"/>
-      <c r="B51" s="22" t="s">
+      <c r="A51" s="8"/>
+      <c r="B51" s="9" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A52" s="21"/>
-      <c r="B52" s="22" t="s">
+      <c r="A52" s="8"/>
+      <c r="B52" s="9" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A53" s="21"/>
-      <c r="B53" s="22" t="s">
+      <c r="A53" s="8"/>
+      <c r="B53" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A54" s="21"/>
-      <c r="B54" s="22" t="s">
+      <c r="A54" s="8"/>
+      <c r="B54" s="9" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A55" s="21"/>
-      <c r="B55" s="22" t="s">
+      <c r="A55" s="8"/>
+      <c r="B55" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A56" s="23"/>
-      <c r="B56" s="24" t="s">
+      <c r="A56" s="10"/>
+      <c r="B56" s="11" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A18:B18"/>
     <mergeCell ref="E18:J23"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A26:B26"/>
@@ -3506,6 +3488,12 @@
     <mergeCell ref="E5:J6"/>
     <mergeCell ref="E9:J11"/>
     <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A18:B18"/>
   </mergeCells>
   <conditionalFormatting sqref="A34:B34">
     <cfRule type="containsText" dxfId="77" priority="22" operator="containsText" text="REVIEW NOT COMPLETE">
@@ -3622,157 +3610,157 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="15"/>
+      <c r="B1" s="2"/>
     </row>
     <row r="2" spans="1:8" ht="78.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="13"/>
+      <c r="B2" s="47"/>
     </row>
     <row r="3" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A3" s="25"/>
+      <c r="A3" s="12"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="59"/>
+      <c r="B4" s="60"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="7" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="15" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25"/>
-      <c r="D7" s="60" t="s">
+      <c r="A7" s="12"/>
+      <c r="D7" s="61" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="60"/>
-      <c r="F7" s="60"/>
-      <c r="G7" s="60"/>
-      <c r="H7" s="60"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="61"/>
+      <c r="H7" s="61"/>
     </row>
     <row r="8" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="30">
+      <c r="B8" s="17">
         <v>1</v>
       </c>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
-      <c r="G8" s="60"/>
-      <c r="H8" s="60"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="61"/>
     </row>
     <row r="9" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="60"/>
-      <c r="G9" s="60"/>
-      <c r="H9" s="60"/>
+      <c r="D9" s="61"/>
+      <c r="E9" s="61"/>
+      <c r="F9" s="61"/>
+      <c r="G9" s="61"/>
+      <c r="H9" s="61"/>
     </row>
     <row r="10" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="30">
+      <c r="B10" s="17">
         <v>1</v>
       </c>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
-      <c r="G10" s="60"/>
-      <c r="H10" s="60"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
     </row>
     <row r="11" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B11" s="31">
+      <c r="B11" s="18">
         <v>46303</v>
       </c>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
     </row>
     <row r="12" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
     </row>
     <row r="13" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="61" t="s">
+      <c r="A13" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="B13" s="61"/>
-      <c r="D13" s="60"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="60"/>
-      <c r="H13" s="60"/>
+      <c r="B13" s="62"/>
+      <c r="D13" s="61"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="61"/>
+      <c r="H13" s="61"/>
     </row>
     <row r="14" spans="1:8" ht="65.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="62" t="s">
+      <c r="A14" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="62"/>
+      <c r="B14" s="63"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="33" t="s">
+      <c r="A16" s="20" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="63" t="s">
+      <c r="A17" s="59" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="63"/>
+      <c r="B17" s="59"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="33" t="s">
+      <c r="A19" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="29" t="s">
+      <c r="A20" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="30" t="s">
+      <c r="B20" s="17" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="29" t="s">
+      <c r="A21" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B21" s="30" t="s">
+      <c r="B21" s="17" t="s">
         <v>59</v>
       </c>
     </row>
@@ -3829,388 +3817,388 @@
   <cols>
     <col min="1" max="1" width="74.5" customWidth="1"/>
     <col min="2" max="2" width="20.6640625" customWidth="1"/>
-    <col min="3" max="3" width="20.6640625" style="34" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" style="21" customWidth="1"/>
     <col min="4" max="4" width="60.6640625" customWidth="1"/>
     <col min="5" max="6" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="15"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="47" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
     </row>
     <row r="3" spans="1:4" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="48" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="25"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="36"/>
+      <c r="A4" s="12"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="23"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="37"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="24"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="38"/>
+      <c r="C6" s="50"/>
+      <c r="D6" s="25"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="39"/>
+      <c r="C7" s="51"/>
+      <c r="D7" s="26"/>
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
+      <c r="A8" s="12"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B9" s="40" t="s">
+      <c r="B9" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="40" t="s">
+      <c r="C9" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="40" t="s">
+      <c r="D9" s="27" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="40"/>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="41"/>
-      <c r="D11" s="42"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="29"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="43" t="s">
+      <c r="A14" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="B14" s="41" t="s">
+      <c r="B14" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="41"/>
-      <c r="D14" s="42"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="29"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B15" s="34"/>
+      <c r="B15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="B16" s="40"/>
-      <c r="C16" s="40"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="B17" s="41" t="s">
+      <c r="B17" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="41"/>
-      <c r="D17" s="42"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="29"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="43" t="s">
+      <c r="A18" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="41" t="s">
+      <c r="B18" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="41"/>
-      <c r="D18" s="42"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="29"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="43" t="s">
+      <c r="A19" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="B19" s="41" t="s">
+      <c r="B19" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="41"/>
-      <c r="D19" s="42"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="29"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="43" t="s">
+      <c r="A20" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="B20" s="41" t="s">
+      <c r="B20" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="41"/>
-      <c r="D20" s="42"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="29"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="B21" s="41" t="s">
+      <c r="B21" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="42"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="29"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="41" t="s">
+      <c r="B22" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="41"/>
-      <c r="D22" s="42"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="29"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="43" t="s">
+      <c r="A23" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="41" t="s">
+      <c r="B23" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="41"/>
-      <c r="D23" s="42"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="29"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="43"/>
-      <c r="B24" s="43"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
+      <c r="A24" s="30"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="43"/>
+      <c r="A25" s="30"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="32" t="s">
+      <c r="A26" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="B26" s="40"/>
-      <c r="C26" s="40"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="B27" s="41" t="s">
+      <c r="B27" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C27" s="41"/>
-      <c r="D27" s="42"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="29"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B28" s="34"/>
+      <c r="B28" s="21"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="32" t="s">
+      <c r="A29" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="B29" s="44"/>
-      <c r="C29" s="44"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="43" t="s">
+      <c r="A30" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="B30" s="41" t="s">
+      <c r="B30" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="42"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="29"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="43" t="s">
+      <c r="A31" s="30" t="s">
         <v>82</v>
       </c>
-      <c r="B31" s="41" t="s">
+      <c r="B31" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C31" s="41"/>
-      <c r="D31" s="42"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="29"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B32" s="34"/>
+      <c r="B32" s="21"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="32" t="s">
+      <c r="A33" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="B33" s="44"/>
-      <c r="C33" s="44"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="31"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="43" t="s">
+      <c r="A34" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="B34" s="41" t="s">
+      <c r="B34" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="C34" s="41"/>
-      <c r="D34" s="42"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="29"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="43" t="s">
+      <c r="A35" s="30" t="s">
         <v>86</v>
       </c>
-      <c r="B35" s="41" t="s">
+      <c r="B35" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="C35" s="41"/>
-      <c r="D35" s="42"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="29"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="43" t="s">
+      <c r="A36" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="B36" s="41" t="s">
+      <c r="B36" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="C36" s="41"/>
-      <c r="D36" s="42"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="29"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="43" t="s">
+      <c r="A37" s="30" t="s">
         <v>88</v>
       </c>
-      <c r="B37" s="41" t="s">
+      <c r="B37" s="28" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="41"/>
-      <c r="D37" s="42"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="29"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="43" t="s">
+      <c r="A38" s="30" t="s">
         <v>90</v>
       </c>
-      <c r="B38" s="41" t="s">
+      <c r="B38" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="C38" s="41"/>
-      <c r="D38" s="42"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="29"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="43" t="s">
+      <c r="A39" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="B39" s="41" t="s">
+      <c r="B39" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="42"/>
+      <c r="C39" s="28"/>
+      <c r="D39" s="29"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B40" s="34"/>
+      <c r="B40" s="21"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="32" t="s">
+      <c r="A41" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="B41" s="34"/>
+      <c r="B41" s="21"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="43" t="s">
+      <c r="A42" s="30" t="s">
         <v>93</v>
       </c>
-      <c r="B42" s="41" t="s">
+      <c r="B42" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C42" s="41"/>
-      <c r="D42" s="42"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="29"/>
     </row>
     <row r="43" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A43" s="45" t="s">
+      <c r="A43" s="32" t="s">
         <v>94</v>
       </c>
-      <c r="B43" s="46" t="s">
+      <c r="B43" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="C43" s="46"/>
-      <c r="D43" s="47"/>
+      <c r="C43" s="33"/>
+      <c r="D43" s="34"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B44" s="34"/>
+      <c r="B44" s="21"/>
     </row>
     <row r="46" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="8" t="s">
+      <c r="A46" s="46" t="s">
         <v>95</v>
       </c>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
+      <c r="B46" s="46"/>
+      <c r="C46" s="46"/>
+      <c r="D46" s="46"/>
     </row>
     <row r="47" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="8"/>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
+      <c r="A47" s="46"/>
+      <c r="B47" s="46"/>
+      <c r="C47" s="46"/>
+      <c r="D47" s="46"/>
     </row>
     <row r="48" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="8"/>
-      <c r="B48" s="8"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
+      <c r="A48" s="46"/>
+      <c r="B48" s="46"/>
+      <c r="C48" s="46"/>
+      <c r="D48" s="46"/>
     </row>
     <row r="49" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="8"/>
-      <c r="B49" s="8"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
+      <c r="A49" s="46"/>
+      <c r="B49" s="46"/>
+      <c r="C49" s="46"/>
+      <c r="D49" s="46"/>
     </row>
     <row r="75" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E75" t="s">
@@ -4354,241 +4342,237 @@
   <cols>
     <col min="1" max="1" width="72.5" customWidth="1"/>
     <col min="2" max="2" width="19.1640625" customWidth="1"/>
-    <col min="3" max="3" width="20.6640625" style="34" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" style="21" customWidth="1"/>
     <col min="4" max="4" width="60.6640625" customWidth="1"/>
     <col min="5" max="6" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="15"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="47" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
     </row>
     <row r="3" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="48" t="s">
         <v>99</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
     </row>
     <row r="4" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A4" s="25"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="36"/>
+      <c r="A4" s="12"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="23"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="37"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="24"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="48"/>
+      <c r="C6" s="50"/>
+      <c r="D6" s="35"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="49"/>
+      <c r="C7" s="51"/>
+      <c r="D7" s="36"/>
     </row>
     <row r="8" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="36"/>
+      <c r="A8" s="12"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="23"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B9" s="40" t="s">
+      <c r="B9" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="40" t="s">
+      <c r="C9" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="40" t="s">
+      <c r="D9" s="27" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="B10" s="33"/>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="30" t="s">
         <v>101</v>
       </c>
-      <c r="B11" s="41" t="s">
-        <v>230</v>
-      </c>
-      <c r="C11" s="41"/>
-      <c r="D11" s="42" t="s">
-        <v>229</v>
-      </c>
+      <c r="B11" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="28"/>
+      <c r="D11" s="29"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="50" t="s">
+      <c r="A14" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="B14" s="41" t="s">
+      <c r="B14" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="41"/>
-      <c r="D14" s="42"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="29"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="33" t="s">
+      <c r="A16" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="B16" s="33"/>
-      <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="B17" s="41" t="s">
+      <c r="B17" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="41"/>
-      <c r="D17" s="42"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="29"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="43" t="s">
+      <c r="A18" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="B18" s="41" t="s">
+      <c r="B18" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="41"/>
-      <c r="D18" s="42"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="29"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="43" t="s">
+      <c r="A19" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="B19" s="41" t="s">
+      <c r="B19" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="41"/>
-      <c r="D19" s="42"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="29"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="43" t="s">
+      <c r="A20" s="30" t="s">
         <v>108</v>
       </c>
-      <c r="B20" s="41" t="s">
-        <v>230</v>
-      </c>
-      <c r="C20" s="41"/>
-      <c r="D20" s="42" t="s">
-        <v>231</v>
-      </c>
+      <c r="B20" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="28"/>
+      <c r="D20" s="29"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="30" t="s">
         <v>109</v>
       </c>
-      <c r="B21" s="41" t="s">
+      <c r="B21" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="41"/>
-      <c r="D21" s="42"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="29"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="32" t="s">
+      <c r="A23" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="B23" s="32"/>
-      <c r="C23" s="40"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="27"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="43" t="s">
+      <c r="A24" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="B24" s="41" t="s">
+      <c r="B24" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="41"/>
-      <c r="D24" s="42"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="29"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="43" t="s">
+      <c r="A25" s="30" t="s">
         <v>112</v>
       </c>
-      <c r="B25" s="41" t="s">
+      <c r="B25" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="41"/>
-      <c r="D25" s="42"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="29"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="43" t="s">
+      <c r="A26" s="30" t="s">
         <v>113</v>
       </c>
-      <c r="B26" s="41" t="s">
+      <c r="B26" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="41"/>
-      <c r="D26" s="42"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="29"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="B27" s="41" t="s">
+      <c r="B27" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C27" s="41"/>
-      <c r="D27" s="42"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="29"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="43" t="s">
+      <c r="A28" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="B28" s="41" t="s">
+      <c r="B28" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C28" s="41"/>
-      <c r="D28" s="42"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="29"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
@@ -4596,102 +4580,104 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="32" t="s">
+      <c r="A30" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="B30" s="32"/>
-      <c r="C30" s="44"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="31"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="43" t="s">
+      <c r="A31" s="30" t="s">
         <v>118</v>
       </c>
-      <c r="B31" s="41"/>
-      <c r="C31" s="41"/>
-      <c r="D31" s="42"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="29"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="43" t="s">
+      <c r="A32" s="30" t="s">
         <v>119</v>
       </c>
-      <c r="B32" s="41"/>
-      <c r="C32" s="41"/>
-      <c r="D32" s="42"/>
+      <c r="B32" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="C32" s="28"/>
+      <c r="D32" s="29"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="43" t="s">
+      <c r="A33" s="30" t="s">
         <v>120</v>
       </c>
-      <c r="B33" s="41"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="42"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="29"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="32" t="s">
+      <c r="A35" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="B35" s="44"/>
-      <c r="C35" s="44"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="31"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="43" t="s">
+      <c r="A36" s="30" t="s">
         <v>122</v>
       </c>
-      <c r="B36" s="41" t="s">
+      <c r="B36" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C36" s="41"/>
-      <c r="D36" s="42"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="29"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="43" t="s">
+      <c r="A37" s="30" t="s">
         <v>123</v>
       </c>
-      <c r="B37" s="41"/>
-      <c r="C37" s="41"/>
-      <c r="D37" s="42"/>
+      <c r="B37" s="28"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="29"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="43" t="s">
+      <c r="A38" s="30" t="s">
         <v>124</v>
       </c>
-      <c r="B38" s="41"/>
-      <c r="C38" s="41"/>
-      <c r="D38" s="42"/>
+      <c r="B38" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="C38" s="28"/>
+      <c r="D38" s="29"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="43" t="s">
+      <c r="A39" s="30" t="s">
         <v>125</v>
       </c>
-      <c r="B39" s="41" t="s">
-        <v>230</v>
-      </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="42" t="s">
-        <v>232</v>
-      </c>
+      <c r="B39" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="C39" s="28"/>
+      <c r="D39" s="29"/>
     </row>
     <row r="42" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="46" t="s">
         <v>126</v>
       </c>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
+      <c r="C42" s="46"/>
+      <c r="D42" s="46"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B43" s="8"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="8"/>
+      <c r="B43" s="46"/>
+      <c r="C43" s="46"/>
+      <c r="D43" s="46"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
+      <c r="B44" s="46"/>
+      <c r="C44" s="46"/>
+      <c r="D44" s="46"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
+      <c r="B45" s="46"/>
+      <c r="C45" s="46"/>
+      <c r="D45" s="46"/>
     </row>
     <row r="58" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F58" t="s">
@@ -4812,167 +4798,167 @@
   <cols>
     <col min="1" max="1" width="67.33203125" customWidth="1"/>
     <col min="2" max="2" width="20.6640625" customWidth="1"/>
-    <col min="3" max="3" width="20.6640625" style="34" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" style="21" customWidth="1"/>
     <col min="4" max="4" width="60.6640625" customWidth="1"/>
     <col min="5" max="6" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="15"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="47" t="s">
         <v>129</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
     </row>
     <row r="3" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A3" s="25"/>
-      <c r="B3" s="25"/>
-      <c r="C3" s="36"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="23"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="37"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="24"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="48"/>
+      <c r="C5" s="50"/>
+      <c r="D5" s="35"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="49"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="36"/>
     </row>
     <row r="7" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A7" s="25"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
+      <c r="A7" s="12"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
     </row>
     <row r="8" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A8" s="25"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
+      <c r="A8" s="12"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B9" s="40" t="s">
+      <c r="B9" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="40" t="s">
+      <c r="C9" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="40" t="s">
+      <c r="D9" s="27" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="B10" s="40"/>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="30" t="s">
         <v>131</v>
       </c>
-      <c r="B11" s="41"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="51"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="38"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="30" t="s">
         <v>132</v>
       </c>
-      <c r="B12" s="41"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="51"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="38"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="43" t="s">
+      <c r="A13" s="30" t="s">
         <v>133</v>
       </c>
-      <c r="B13" s="41"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="51"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="38"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="43" t="s">
+      <c r="A14" s="30" t="s">
         <v>134</v>
       </c>
-      <c r="B14" s="41"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="51"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="38"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B15" s="34"/>
+      <c r="B15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="B16" s="40"/>
-      <c r="C16" s="40"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="30" t="s">
         <v>136</v>
       </c>
-      <c r="B17" s="41"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="51"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="38"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="43" t="s">
+      <c r="A18" s="30" t="s">
         <v>137</v>
       </c>
-      <c r="B18" s="41"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="51"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="38"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="33" t="s">
+      <c r="A20" s="20" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="30" t="s">
         <v>139</v>
       </c>
-      <c r="B21" s="41"/>
-      <c r="C21" s="41"/>
-      <c r="D21" s="51"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="38"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="30" t="s">
         <v>140</v>
       </c>
-      <c r="B22" s="41"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="51"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="38"/>
     </row>
     <row r="25" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="26" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -5063,15 +5049,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
     </row>
     <row r="2" spans="1:7" ht="78" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="64" t="s">
@@ -5085,47 +5071,47 @@
       <c r="G2" s="64"/>
     </row>
     <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="52"/>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="53"/>
-      <c r="G3" s="53"/>
+      <c r="A3" s="39"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="37"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="24"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="48"/>
+      <c r="C5" s="35"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="49"/>
+      <c r="C6" s="36"/>
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="52"/>
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="53"/>
-      <c r="E7" s="53"/>
-      <c r="F7" s="53"/>
-      <c r="G7" s="53"/>
+      <c r="A7" s="39"/>
+      <c r="B7" s="40"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="40"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -5197,7 +5183,7 @@
       <c r="D12" t="s">
         <v>158</v>
       </c>
-      <c r="E12" s="55" t="s">
+      <c r="E12" s="42" t="s">
         <v>163</v>
       </c>
     </row>
@@ -5214,7 +5200,7 @@
       <c r="D13" t="s">
         <v>153</v>
       </c>
-      <c r="E13" s="55" t="s">
+      <c r="E13" s="42" t="s">
         <v>166</v>
       </c>
     </row>
@@ -5231,7 +5217,7 @@
       <c r="D14" t="s">
         <v>158</v>
       </c>
-      <c r="E14" s="55" t="s">
+      <c r="E14" s="42" t="s">
         <v>169</v>
       </c>
     </row>
@@ -5265,7 +5251,7 @@
       <c r="D16" t="s">
         <v>153</v>
       </c>
-      <c r="E16" s="55" t="s">
+      <c r="E16" s="42" t="s">
         <v>176</v>
       </c>
     </row>
@@ -5282,7 +5268,7 @@
       <c r="D17" t="s">
         <v>158</v>
       </c>
-      <c r="E17" s="55" t="s">
+      <c r="E17" s="42" t="s">
         <v>179</v>
       </c>
     </row>
@@ -5299,7 +5285,7 @@
       <c r="D18" t="s">
         <v>158</v>
       </c>
-      <c r="E18" s="55" t="s">
+      <c r="E18" s="42" t="s">
         <v>183</v>
       </c>
     </row>
@@ -5316,12 +5302,12 @@
       <c r="D19" t="s">
         <v>187</v>
       </c>
-      <c r="E19" s="55" t="s">
+      <c r="E19" s="42" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="E20" s="56" t="s">
+      <c r="E20" s="43" t="s">
         <v>189</v>
       </c>
     </row>
@@ -5409,12 +5395,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="65" t="s">
@@ -5425,29 +5411,29 @@
       <c r="D2" s="65"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="37"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="24"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="48"/>
+      <c r="C5" s="35"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="49"/>
+      <c r="C6" s="36"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -5464,7 +5450,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="57">
+      <c r="A10" s="44">
         <v>36526</v>
       </c>
       <c r="B10" t="s">
@@ -5540,16 +5526,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="20" t="s">
         <v>200</v>
       </c>
-      <c r="C1" s="33" t="s">
+      <c r="C1" s="20" t="s">
         <v>201</v>
       </c>
-      <c r="D1" s="33" t="s">
+      <c r="D1" s="20" t="s">
         <v>202</v>
       </c>
       <c r="E1" t="s">
@@ -5572,10 +5558,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="45" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="45" t="s">
         <v>44</v>
       </c>
       <c r="C2" t="s">
@@ -5604,10 +5590,10 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="58" t="s">
+      <c r="A3" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="58" t="s">
+      <c r="B3" s="45" t="s">
         <v>46</v>
       </c>
       <c r="C3" t="s">
@@ -5636,7 +5622,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="45" t="s">
         <v>220</v>
       </c>
       <c r="C4" t="s">

</xml_diff>

<commit_message>
PCB AND SCHEMATIC DONEZO
</commit_message>
<xml_diff>
--- a/DRS Project/Design Files/Electrical System/DDR.xlsx
+++ b/DRS Project/Design Files/Electrical System/DDR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/theodevos-vernes/Documents/GitHub/ENGG2200/DRS Project/Design Files/Electrical System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0697B14B-9776-D043-8AFF-3FF1E82B4DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F80D2A-F072-E449-B61B-5D2DD2D4F0E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="600" windowWidth="28800" windowHeight="17400" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DETAILED DESIGN REVIEW" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="241">
   <si>
     <t>PCB DDR</t>
   </si>
@@ -1181,6 +1181,36 @@
   </si>
   <si>
     <t>This board is required to receive power and a CAN signal from the vehicle/testbench. This board must regulate the power received into voltages appropriate for driving a servo motor, a Teensy 4.0 microcontroller and a CAN transceiver. This board must also communicate with the vehicle/testbench via CAN protocol in order to control a moveable aero device via servo motor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bold titles </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change abbreviations into clear explanations </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add capacitor to voltage regulation (Vin), </t>
+  </si>
+  <si>
+    <t xml:space="preserve">12V protected TP, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teensy Datasheet, SS54 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adds blocks around circuits to clearly label components </t>
+  </si>
+  <si>
+    <t>Maybe consider MOLEX connector for servo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remopve TPX from all test points, do CAN H and CAN L for TPs, Maybe consider row of test points for neatness </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Double check 3.3V trace on CAN IC, CAN H and CAN L run next to each other </t>
+  </si>
+  <si>
+    <t>Dom Brymora</t>
   </si>
 </sst>
 </file>
@@ -1696,7 +1726,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="2" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1791,8 +1821,14 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1806,6 +1842,15 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1813,18 +1858,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="2" applyAlignment="1" applyProtection="1">
@@ -1839,15 +1872,13 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="2" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Excel Built-in Input" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
@@ -3050,20 +3081,20 @@
       <c r="B1" s="2"/>
     </row>
     <row r="2" spans="1:10" ht="80.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="46"/>
+      <c r="B2" s="47"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E3" s="55" t="s">
+      <c r="E3" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="53"/>
+      <c r="I3" s="53"/>
+      <c r="J3" s="53"/>
     </row>
     <row r="4" spans="1:10" ht="21" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
@@ -3072,12 +3103,12 @@
       <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="53"/>
     </row>
     <row r="5" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -3086,14 +3117,14 @@
       <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="56" t="s">
+      <c r="E5" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
-      <c r="H5" s="56"/>
-      <c r="I5" s="56"/>
-      <c r="J5" s="56"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="54"/>
     </row>
     <row r="6" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -3102,62 +3133,66 @@
       <c r="B6" s="4">
         <v>1</v>
       </c>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="56"/>
-      <c r="I6" s="56"/>
-      <c r="J6" s="56"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="54"/>
     </row>
     <row r="8" spans="1:10" ht="21" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="4"/>
+      <c r="B8" s="65">
+        <v>46311</v>
+      </c>
     </row>
     <row r="9" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="E9" s="54" t="s">
+      <c r="B9" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="E9" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
-      <c r="J9" s="54"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="46"/>
+      <c r="J9" s="46"/>
     </row>
     <row r="10" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="4"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="54"/>
-      <c r="H10" s="54"/>
-      <c r="I10" s="54"/>
-      <c r="J10" s="54"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="46"/>
+      <c r="J10" s="46"/>
     </row>
     <row r="11" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B11" s="4"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="54"/>
-      <c r="I11" s="54"/>
-      <c r="J11" s="54"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="46"/>
+      <c r="I11" s="46"/>
+      <c r="J11" s="46"/>
     </row>
     <row r="12" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="57" t="s">
+      <c r="A12" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="57"/>
+      <c r="B12" s="55"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
@@ -3172,10 +3207,10 @@
       <c r="J13" s="5"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="52" t="s">
+      <c r="A14" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="52"/>
+      <c r="B14" s="57"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
@@ -3192,7 +3227,7 @@
       </c>
       <c r="B16" s="7" t="str">
         <f>'PCB Design Intent'!B6</f>
-        <v>NO</v>
+        <v>YES</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
@@ -3200,18 +3235,18 @@
       <c r="B17" s="9"/>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="50" t="s">
+      <c r="A18" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="50"/>
-      <c r="E18" s="54" t="s">
+      <c r="B18" s="52"/>
+      <c r="E18" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="F18" s="54"/>
-      <c r="G18" s="54"/>
-      <c r="H18" s="54"/>
-      <c r="I18" s="54"/>
-      <c r="J18" s="54"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="46"/>
+      <c r="I18" s="46"/>
+      <c r="J18" s="46"/>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
@@ -3221,12 +3256,12 @@
         <f>'Schematic Review'!B6</f>
         <v>YES</v>
       </c>
-      <c r="E19" s="54"/>
-      <c r="F19" s="54"/>
-      <c r="G19" s="54"/>
-      <c r="H19" s="54"/>
-      <c r="I19" s="54"/>
-      <c r="J19" s="54"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="46"/>
     </row>
     <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
@@ -3234,36 +3269,36 @@
       </c>
       <c r="B20" s="7" t="str">
         <f>'Schematic Review'!B7</f>
-        <v>NO</v>
-      </c>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="54"/>
-      <c r="H20" s="54"/>
-      <c r="I20" s="54"/>
-      <c r="J20" s="54"/>
+        <v>YES</v>
+      </c>
+      <c r="E20" s="46"/>
+      <c r="F20" s="46"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="46"/>
+      <c r="I20" s="46"/>
+      <c r="J20" s="46"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="6"/>
       <c r="B21" s="9"/>
-      <c r="E21" s="54"/>
-      <c r="F21" s="54"/>
-      <c r="G21" s="54"/>
-      <c r="H21" s="54"/>
-      <c r="I21" s="54"/>
-      <c r="J21" s="54"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="46"/>
+      <c r="J21" s="46"/>
     </row>
     <row r="22" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="50" t="s">
+      <c r="A22" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="50"/>
-      <c r="E22" s="54"/>
-      <c r="F22" s="54"/>
-      <c r="G22" s="54"/>
-      <c r="H22" s="54"/>
-      <c r="I22" s="54"/>
-      <c r="J22" s="54"/>
+      <c r="B22" s="52"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="46"/>
+      <c r="H22" s="46"/>
+      <c r="I22" s="46"/>
+      <c r="J22" s="46"/>
     </row>
     <row r="23" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
@@ -3273,12 +3308,12 @@
         <f>'Layout Review'!B6</f>
         <v>YES</v>
       </c>
-      <c r="E23" s="54"/>
-      <c r="F23" s="54"/>
-      <c r="G23" s="54"/>
-      <c r="H23" s="54"/>
-      <c r="I23" s="54"/>
-      <c r="J23" s="54"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
+      <c r="I23" s="46"/>
+      <c r="J23" s="46"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
@@ -3286,7 +3321,7 @@
       </c>
       <c r="B24" s="7" t="str">
         <f>'Layout Review'!B7</f>
-        <v>NO</v>
+        <v>YES</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -3294,10 +3329,10 @@
       <c r="B25" s="9"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="50" t="s">
+      <c r="A26" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="50"/>
+      <c r="B26" s="52"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
@@ -3322,10 +3357,10 @@
       <c r="B29" s="9"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" s="50" t="s">
+      <c r="A30" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="B30" s="50"/>
+      <c r="B30" s="52"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
@@ -3350,23 +3385,23 @@
       <c r="B33" s="9"/>
     </row>
     <row r="34" spans="1:2" ht="26" x14ac:dyDescent="0.3">
-      <c r="A34" s="51" t="str">
+      <c r="A34" s="56" t="str">
         <f>IF((AND(B15="YES",B16="YES",B19="YES",B20="YES",B23="YES",B24="YES",B27="YES",B28="YES",B31="YES",B32="YES")), "PCB REVIEWED AND READY FOR MANUFACTURE", "REVIEW NOT COMPLETE")</f>
         <v>REVIEW NOT COMPLETE</v>
       </c>
-      <c r="B34" s="51"/>
+      <c r="B34" s="56"/>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" s="52" t="s">
+      <c r="A37" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="B37" s="52"/>
+      <c r="B37" s="57"/>
     </row>
     <row r="38" spans="1:2" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="53" t="s">
+      <c r="A38" s="58" t="s">
         <v>24</v>
       </c>
-      <c r="B38" s="53"/>
+      <c r="B38" s="58"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="8"/>
@@ -3478,6 +3513,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A18:B18"/>
     <mergeCell ref="E18:J23"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A26:B26"/>
@@ -3486,12 +3527,6 @@
     <mergeCell ref="E5:J6"/>
     <mergeCell ref="E9:J11"/>
     <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A18:B18"/>
   </mergeCells>
   <conditionalFormatting sqref="A34:B34">
     <cfRule type="containsText" dxfId="77" priority="22" operator="containsText" text="REVIEW NOT COMPLETE">
@@ -3614,19 +3649,19 @@
       <c r="B1" s="2"/>
     </row>
     <row r="2" spans="1:8" ht="78.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="46"/>
+      <c r="B2" s="47"/>
     </row>
     <row r="3" spans="1:8" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="12"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="59"/>
+      <c r="B4" s="60"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
@@ -3641,18 +3676,18 @@
         <v>46</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12"/>
-      <c r="D7" s="54" t="s">
+      <c r="D7" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
-      <c r="H7" s="54"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="46"/>
+      <c r="H7" s="46"/>
     </row>
     <row r="8" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="16" t="s">
@@ -3661,11 +3696,11 @@
       <c r="B8" s="17">
         <v>1</v>
       </c>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="54"/>
-      <c r="H8" s="54"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="46"/>
     </row>
     <row r="9" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="16" t="s">
@@ -3674,11 +3709,11 @@
       <c r="B9" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46"/>
     </row>
     <row r="10" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="16" t="s">
@@ -3687,11 +3722,11 @@
       <c r="B10" s="17">
         <v>1</v>
       </c>
-      <c r="D10" s="54"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="54"/>
-      <c r="H10" s="54"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
     </row>
     <row r="11" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="16" t="s">
@@ -3700,35 +3735,35 @@
       <c r="B11" s="18">
         <v>46303</v>
       </c>
-      <c r="D11" s="54"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="54"/>
+      <c r="D11" s="46"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="46"/>
     </row>
     <row r="12" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D12" s="54"/>
-      <c r="E12" s="54"/>
-      <c r="F12" s="54"/>
-      <c r="G12" s="54"/>
-      <c r="H12" s="54"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="46"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="46"/>
     </row>
     <row r="13" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="60" t="s">
+      <c r="A13" s="61" t="s">
         <v>51</v>
       </c>
-      <c r="B13" s="60"/>
-      <c r="D13" s="54"/>
-      <c r="E13" s="54"/>
-      <c r="F13" s="54"/>
-      <c r="G13" s="54"/>
-      <c r="H13" s="54"/>
+      <c r="B13" s="61"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="46"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="46"/>
     </row>
     <row r="14" spans="1:8" ht="65.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="61" t="s">
+      <c r="A14" s="62" t="s">
         <v>230</v>
       </c>
-      <c r="B14" s="61"/>
+      <c r="B14" s="62"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="20" t="s">
@@ -3736,10 +3771,10 @@
       </c>
     </row>
     <row r="17" spans="1:2" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="58" t="s">
+      <c r="A17" s="59" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="58"/>
+      <c r="B17" s="59"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="20" t="s">
@@ -3829,20 +3864,20 @@
       <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
     </row>
     <row r="3" spans="1:4" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12"/>
@@ -3850,31 +3885,31 @@
       <c r="C4" s="23"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="47" t="s">
+      <c r="A5" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
       <c r="D5" s="24"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="48" t="s">
-        <v>45</v>
-      </c>
-      <c r="C6" s="48"/>
+      <c r="B6" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="50"/>
       <c r="D6" s="25"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="49" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="49"/>
+      <c r="B7" s="51" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="51"/>
       <c r="D7" s="26"/>
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3908,7 +3943,9 @@
       <c r="B11" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="28"/>
+      <c r="C11" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D11" s="29"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -3931,7 +3968,9 @@
       <c r="B14" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="28"/>
+      <c r="C14" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D14" s="29"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -3951,8 +3990,12 @@
       <c r="B17" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="29"/>
+      <c r="C17" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>231</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="30" t="s">
@@ -3961,8 +4004,12 @@
       <c r="B18" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="28"/>
-      <c r="D18" s="29"/>
+      <c r="C18" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="29" t="s">
+        <v>231</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="30" t="s">
@@ -3971,8 +4018,12 @@
       <c r="B19" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="29"/>
+      <c r="C19" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" s="29" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="30" t="s">
@@ -3981,8 +4032,12 @@
       <c r="B20" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="28"/>
-      <c r="D20" s="29"/>
+      <c r="C20" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="30" t="s">
@@ -3991,7 +4046,9 @@
       <c r="B21" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="28"/>
+      <c r="C21" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D21" s="29"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -4001,7 +4058,9 @@
       <c r="B22" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="28"/>
+      <c r="C22" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D22" s="29"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -4011,8 +4070,12 @@
       <c r="B23" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="28"/>
-      <c r="D23" s="29"/>
+      <c r="C23" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="29" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="30"/>
@@ -4037,8 +4100,12 @@
       <c r="B27" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C27" s="28"/>
-      <c r="D27" s="29"/>
+      <c r="C27" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="29" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B28" s="21"/>
@@ -4057,7 +4124,9 @@
       <c r="B30" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C30" s="28"/>
+      <c r="C30" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D30" s="29"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -4067,7 +4136,9 @@
       <c r="B31" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C31" s="28"/>
+      <c r="C31" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D31" s="29"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
@@ -4087,7 +4158,9 @@
       <c r="B34" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="C34" s="28"/>
+      <c r="C34" s="28" t="s">
+        <v>84</v>
+      </c>
       <c r="D34" s="29"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
@@ -4097,7 +4170,9 @@
       <c r="B35" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="C35" s="28"/>
+      <c r="C35" s="28" t="s">
+        <v>84</v>
+      </c>
       <c r="D35" s="29"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
@@ -4107,7 +4182,9 @@
       <c r="B36" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="C36" s="28"/>
+      <c r="C36" s="28" t="s">
+        <v>84</v>
+      </c>
       <c r="D36" s="29"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
@@ -4117,7 +4194,9 @@
       <c r="B37" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="C37" s="28"/>
+      <c r="C37" s="28" t="s">
+        <v>88</v>
+      </c>
       <c r="D37" s="29"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
@@ -4127,7 +4206,9 @@
       <c r="B38" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="C38" s="28"/>
+      <c r="C38" s="28" t="s">
+        <v>84</v>
+      </c>
       <c r="D38" s="29"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
@@ -4137,7 +4218,9 @@
       <c r="B39" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="C39" s="28"/>
+      <c r="C39" s="28" t="s">
+        <v>84</v>
+      </c>
       <c r="D39" s="29"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
@@ -4156,7 +4239,9 @@
       <c r="B42" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C42" s="28"/>
+      <c r="C42" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D42" s="29"/>
     </row>
     <row r="43" spans="1:4" ht="32" x14ac:dyDescent="0.2">
@@ -4166,37 +4251,39 @@
       <c r="B43" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="C43" s="33"/>
+      <c r="C43" s="33" t="s">
+        <v>45</v>
+      </c>
       <c r="D43" s="34"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B44" s="21"/>
     </row>
     <row r="46" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="54" t="s">
+      <c r="A46" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="B46" s="54"/>
-      <c r="C46" s="54"/>
-      <c r="D46" s="54"/>
+      <c r="B46" s="46"/>
+      <c r="C46" s="46"/>
+      <c r="D46" s="46"/>
     </row>
     <row r="47" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="54"/>
-      <c r="B47" s="54"/>
-      <c r="C47" s="54"/>
-      <c r="D47" s="54"/>
+      <c r="A47" s="46"/>
+      <c r="B47" s="46"/>
+      <c r="C47" s="46"/>
+      <c r="D47" s="46"/>
     </row>
     <row r="48" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="54"/>
-      <c r="B48" s="54"/>
-      <c r="C48" s="54"/>
-      <c r="D48" s="54"/>
+      <c r="A48" s="46"/>
+      <c r="B48" s="46"/>
+      <c r="C48" s="46"/>
+      <c r="D48" s="46"/>
     </row>
     <row r="49" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="54"/>
-      <c r="B49" s="54"/>
-      <c r="C49" s="54"/>
-      <c r="D49" s="54"/>
+      <c r="A49" s="46"/>
+      <c r="B49" s="46"/>
+      <c r="C49" s="46"/>
+      <c r="D49" s="46"/>
     </row>
     <row r="75" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E75" t="s">
@@ -4354,20 +4441,20 @@
       <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="47" t="s">
         <v>97</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
     </row>
     <row r="3" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="48" t="s">
         <v>98</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
     </row>
     <row r="4" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="12"/>
@@ -4375,31 +4462,31 @@
       <c r="C4" s="23"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="47" t="s">
+      <c r="A5" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
       <c r="D5" s="24"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="48" t="s">
-        <v>45</v>
-      </c>
-      <c r="C6" s="48"/>
+      <c r="B6" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="50"/>
       <c r="D6" s="35"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="49" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="49"/>
+      <c r="B7" s="51" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="51"/>
       <c r="D7" s="36"/>
     </row>
     <row r="8" spans="1:4" ht="19" x14ac:dyDescent="0.25">
@@ -4433,7 +4520,9 @@
       <c r="B11" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="28"/>
+      <c r="C11" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D11" s="29"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -4450,7 +4539,9 @@
       <c r="B14" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="28"/>
+      <c r="C14" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D14" s="29"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -4472,8 +4563,12 @@
       <c r="B17" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="29"/>
+      <c r="C17" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="30" t="s">
@@ -4482,7 +4577,9 @@
       <c r="B18" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="28"/>
+      <c r="C18" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D18" s="29"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -4492,7 +4589,9 @@
       <c r="B19" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="28"/>
+      <c r="C19" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D19" s="29"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -4502,18 +4601,24 @@
       <c r="B20" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="28"/>
+      <c r="C20" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D20" s="29"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="30" t="s">
         <v>108</v>
       </c>
       <c r="B21" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="29"/>
+      <c r="C21" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="29" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="19" t="s">
@@ -4529,8 +4634,12 @@
       <c r="B24" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="28"/>
-      <c r="D24" s="29"/>
+      <c r="C24" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" s="29" t="s">
+        <v>239</v>
+      </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="30" t="s">
@@ -4539,7 +4648,9 @@
       <c r="B25" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="28"/>
+      <c r="C25" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D25" s="29"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -4549,7 +4660,9 @@
       <c r="B26" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="28"/>
+      <c r="C26" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D26" s="29"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -4559,7 +4672,9 @@
       <c r="B27" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C27" s="28"/>
+      <c r="C27" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D27" s="29"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -4569,7 +4684,9 @@
       <c r="B28" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C28" s="28"/>
+      <c r="C28" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D28" s="29"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -4591,8 +4708,12 @@
       <c r="B31" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C31" s="28"/>
-      <c r="D31" s="29"/>
+      <c r="C31" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D31" s="29" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="30" t="s">
@@ -4601,7 +4722,9 @@
       <c r="B32" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C32" s="28"/>
+      <c r="C32" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D32" s="29"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
@@ -4611,7 +4734,9 @@
       <c r="B33" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C33" s="28"/>
+      <c r="C33" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D33" s="29" t="s">
         <v>120</v>
       </c>
@@ -4630,7 +4755,9 @@
       <c r="B36" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C36" s="28"/>
+      <c r="C36" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D36" s="29"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
@@ -4640,7 +4767,9 @@
       <c r="B37" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C37" s="28"/>
+      <c r="C37" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D37" s="29"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
@@ -4650,7 +4779,9 @@
       <c r="B38" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C38" s="28"/>
+      <c r="C38" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D38" s="29"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
@@ -4660,30 +4791,32 @@
       <c r="B39" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C39" s="28"/>
+      <c r="C39" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="D39" s="29"/>
     </row>
     <row r="42" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="54" t="s">
+      <c r="B42" s="46" t="s">
         <v>126</v>
       </c>
-      <c r="C42" s="54"/>
-      <c r="D42" s="54"/>
+      <c r="C42" s="46"/>
+      <c r="D42" s="46"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B43" s="54"/>
-      <c r="C43" s="54"/>
-      <c r="D43" s="54"/>
+      <c r="B43" s="46"/>
+      <c r="C43" s="46"/>
+      <c r="D43" s="46"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B44" s="54"/>
-      <c r="C44" s="54"/>
-      <c r="D44" s="54"/>
+      <c r="B44" s="46"/>
+      <c r="C44" s="46"/>
+      <c r="D44" s="46"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B45" s="54"/>
-      <c r="C45" s="54"/>
-      <c r="D45" s="54"/>
+      <c r="B45" s="46"/>
+      <c r="C45" s="46"/>
+      <c r="D45" s="46"/>
     </row>
     <row r="58" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F58" t="s">
@@ -4818,12 +4951,12 @@
       <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="47" t="s">
         <v>129</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
     </row>
     <row r="3" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="12"/>
@@ -4831,31 +4964,31 @@
       <c r="C3" s="23"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="47"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
       <c r="D4" s="24"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="48"/>
+      <c r="C5" s="50"/>
       <c r="D5" s="35"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="49" t="s">
+      <c r="B6" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="49"/>
+      <c r="C6" s="51"/>
       <c r="D6" s="36"/>
     </row>
     <row r="7" spans="1:4" ht="19" x14ac:dyDescent="0.25">
@@ -5024,7 +5157,7 @@
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0400-000000000000}">
           <x14:formula1>
             <xm:f>'DATA VALIDATION'!$B$2:$B$4</xm:f>
@@ -5098,10 +5231,10 @@
       <c r="G3" s="40"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="47"/>
+      <c r="B4" s="49"/>
       <c r="C4" s="24"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -5429,10 +5562,10 @@
       <c r="D2" s="64"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="47"/>
+      <c r="B4" s="49"/>
       <c r="C4" s="24"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>